<commit_message>
Separate user app from internal RAG evaluation
</commit_message>
<xml_diff>
--- a/docs/찾아봇_IA_갱신본_2026-06-14.xlsx
+++ b/docs/찾아봇_IA_갱신본_2026-06-14.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_개요" sheetId="1" r:id="Rc99767c48cbf40f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_사이트맵" sheetId="2" r:id="R1416970f93124c18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_화면정의" sheetId="3" r:id="Rd48b80089d8f4540"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_사용자흐름" sheetId="4" r:id="R1a8e695871ec49bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_컴포넌트" sheetId="5" r:id="R291b0598569f4290"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_데이터_RAG" sheetId="6" r:id="R4974921f20de46e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_음성접근성" sheetId="7" r:id="R0952f0d2fc7146e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_개발산출물" sheetId="8" r:id="Re384ae0726224e46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_개선과제" sheetId="9" r:id="R01301180b54b4619"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_분류통계" sheetId="10" r:id="Rcf20c1fe9cbc4e38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_개요" sheetId="1" r:id="Rfaeaf8e3dc5e4567"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_사이트맵" sheetId="2" r:id="R2a2cbc25b21841ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_화면정의" sheetId="3" r:id="R0202a119eae547da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_사용자흐름" sheetId="4" r:id="Ree58b3f338c746a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_컴포넌트" sheetId="5" r:id="Rf2abce51ad354c1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_데이터_RAG" sheetId="6" r:id="Rbfe8b9283322424e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_음성접근성" sheetId="7" r:id="R668eedcb06674005"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_개발산출물" sheetId="8" r:id="R403ddb01b1584f58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_개선과제" sheetId="9" r:id="R11b2d27b4e1e4e4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_분류통계" sheetId="10" r:id="R071c743673ca4d08"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -347,10 +347,10 @@
         <x:v>현 개발 상태</x:v>
       </x:c>
       <x:c r="B9" s="14" t="str">
-        <x:v>정적 웹 MVP 구현 완료: 홈/대화/탐색/찜/평가 탭, STT/TTS, 통합 DB 418건, RAG 예비 평가</x:v>
+        <x:v>사용자 앱 구현 완료: 홈/대화/탐색/찜, STT/TTS, 통합 DB 418건. RAG 평가는 내부 admin으로 분리</x:v>
       </x:c>
       <x:c r="C9" s="14" t="str">
-        <x:v>컴퓨터공학과 개발 성과로 제시 가능</x:v>
+        <x:v>컴퓨터공학과 개발 성과와 사용자 중심 IA를 함께 제시 가능</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="43.5" customHeight="1">
@@ -380,7 +380,7 @@
         <x:v>평가 전략</x:v>
       </x:c>
       <x:c r="B12" s="14" t="str">
-        <x:v>15문항 평가셋으로 Top-3 적합도, 분류 적합도, Faithfulness 예비 체크</x:v>
+        <x:v>사용자 화면에는 노출하지 않고, admin에서 15문항 평가셋으로 Top-3 적합도, 분류 적합도, Faithfulness 예비 체크</x:v>
       </x:c>
       <x:c r="C12" s="14" t="str">
         <x:v>지도교수 피드백 반영</x:v>
@@ -628,7 +628,7 @@
     </x:row>
     <x:row r="2" ht="31.5" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>현재 구현된 하단 탭과 주요 하위 기능 기준</x:v>
+        <x:v>사용자 앱은 홈/탐색/찜 중심, 내부 평가는 별도 admin 기준</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str"/>
       <x:c r="C2" s="7" t="str"/>
@@ -866,22 +866,22 @@
     </x:row>
     <x:row r="15" ht="43.5" customHeight="1">
       <x:c r="A15" s="14" t="str">
-        <x:v>평가</x:v>
+        <x:v>내부 관리자</x:v>
       </x:c>
       <x:c r="B15" s="14" t="str">
-        <x:v>RAG 예비 평가</x:v>
+        <x:v>RAG·검색 평가</x:v>
       </x:c>
       <x:c r="C15" s="14" t="str">
-        <x:v>screen-eval / runEval</x:v>
+        <x:v>admin.html / runEval</x:v>
       </x:c>
       <x:c r="D15" s="14" t="str">
-        <x:v>하단 평가</x:v>
+        <x:v>직접 URL 접근</x:v>
       </x:c>
       <x:c r="E15" s="14" t="str">
         <x:v>교수 피드백 기반 검색/근거 충실성 평가</x:v>
       </x:c>
       <x:c r="F15" s="14" t="str">
-        <x:v>구현</x:v>
+        <x:v>구현: 사용자 앱과 분리</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="43.5" customHeight="1">
@@ -1113,28 +1113,28 @@
     </x:row>
     <x:row r="9" ht="43.5" customHeight="1">
       <x:c r="A9" s="14" t="str">
-        <x:v>EVL-01</x:v>
+        <x:v>ADM-01</x:v>
       </x:c>
       <x:c r="B9" s="14" t="str">
-        <x:v>RAG 예비 평가</x:v>
+        <x:v>내부 RAG·검색 평가</x:v>
       </x:c>
       <x:c r="C9" s="14" t="str">
-        <x:v>검색 결과의 적합도와 근거 충실성을 확인</x:v>
+        <x:v>검색 결과의 적합도와 근거 충실성을 내부적으로 확인</x:v>
       </x:c>
       <x:c r="D9" s="14" t="str">
-        <x:v>runEval, evalSummary, evalList</x:v>
+        <x:v>runEval, evalSummary, evalList, downloadEval</x:v>
       </x:c>
       <x:c r="E9" s="14" t="str">
         <x:v>평가 실행 버튼</x:v>
       </x:c>
       <x:c r="F9" s="14" t="str">
-        <x:v>Top-3, 분류, Faithfulness 점수</x:v>
+        <x:v>Top-3, 분류, Faithfulness 점수, JSON 결과</x:v>
       </x:c>
       <x:c r="G9" s="14" t="str">
         <x:v>EVAL_SET 15문항, expected keywords/category</x:v>
       </x:c>
       <x:c r="H9" s="14" t="str">
-        <x:v>보고서용 객관 지표 화면</x:v>
+        <x:v>사용자에게 노출하지 않는 내부 평가 화면</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="43.5" customHeight="1">
@@ -1196,7 +1196,7 @@
     </x:row>
     <x:row r="2" ht="31.5" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>어르신 실사용 흐름과 응급/평가/찜 흐름을 분리</x:v>
+        <x:v>어르신 실사용 흐름과 내부 관리자 평가 흐름을 분리</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str"/>
       <x:c r="C2" s="7" t="str"/>
@@ -1397,19 +1397,19 @@
         <x:v>F-05</x:v>
       </x:c>
       <x:c r="B13" s="14" t="str">
-        <x:v>RAG 예비 평가</x:v>
+        <x:v>내부 RAG 평가</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
-        <x:v>평가 탭에서 15문항 실행</x:v>
+        <x:v>관리자가 /admin.html에서 15문항 실행</x:v>
       </x:c>
       <x:c r="E13" s="14" t="str">
-        <x:v>질문별 Top-3/분류/Faithfulness 계산</x:v>
+        <x:v>질문별 Top-3/분류/Faithfulness 계산 및 JSON 다운로드</x:v>
       </x:c>
       <x:c r="F13" s="14" t="str">
-        <x:v>교수 피드백 반영 지표 확인</x:v>
+        <x:v>사용자 경험과 분리된 평가 지표 확인</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1646,7 +1646,7 @@
         <x:v>평가 카드</x:v>
       </x:c>
       <x:c r="B13" s="14" t="str">
-        <x:v>평가</x:v>
+        <x:v>내부 관리자</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
         <x:v>평가셋 결과 표시</x:v>
@@ -1655,10 +1655,10 @@
         <x:v>통과/검토</x:v>
       </x:c>
       <x:c r="E13" s="14" t="str">
-        <x:v>runEvaluation</x:v>
+        <x:v>admin.js runEvaluation</x:v>
       </x:c>
       <x:c r="F13" s="14" t="str">
-        <x:v>교수 피드백 반영</x:v>
+        <x:v>사용자 화면과 분리된 교수 피드백 반영</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="43.5" customHeight="1">
@@ -2128,99 +2128,127 @@
     </x:row>
     <x:row r="7" ht="43.5" customHeight="1">
       <x:c r="A7" s="14" t="str">
-        <x:v>DB 변환 스크립트</x:v>
+        <x:v>DB 정리본</x:v>
       </x:c>
       <x:c r="B7" s="14" t="str">
-        <x:v>scripts/build_resources.py</x:v>
+        <x:v>docs/db-resource-design.md</x:v>
       </x:c>
       <x:c r="C7" s="14" t="str">
-        <x:v>엑셀 원본을 앱용 JSON으로 재생성</x:v>
+        <x:v>앱용 DB, 원본 DB, 평가셋의 역할 분리</x:v>
       </x:c>
       <x:c r="D7" s="14" t="str">
-        <x:v>데이터 수집 결과를 수동 정리에 그치지 않고 재현 가능한 변환 파이프라인으로 구성하였다.</x:v>
+        <x:v>사용자 추천 DB와 내부 RAG 평가셋을 분리하여 설계하였다.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="43.5" customHeight="1">
       <x:c r="A8" s="14" t="str">
-        <x:v>IA 문서</x:v>
+        <x:v>DB 변환 스크립트</x:v>
       </x:c>
       <x:c r="B8" s="14" t="str">
-        <x:v>docs/ia.md / docs/찾아봇_IA_갱신본.xlsx</x:v>
+        <x:v>scripts/build_resources.py</x:v>
       </x:c>
       <x:c r="C8" s="14" t="str">
-        <x:v>구현 기준 IA 정리</x:v>
+        <x:v>엑셀 원본을 앱용 JSON으로 재생성</x:v>
       </x:c>
       <x:c r="D8" s="14" t="str">
-        <x:v>기획 IA를 개발 구현 기준으로 갱신하였다.</x:v>
+        <x:v>데이터 수집 결과를 수동 정리에 그치지 않고 재현 가능한 변환 파이프라인으로 구성하였다.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="43.5" customHeight="1">
       <x:c r="A9" s="14" t="str">
-        <x:v>RAG 평가 문서</x:v>
+        <x:v>IA 문서</x:v>
       </x:c>
       <x:c r="B9" s="14" t="str">
-        <x:v>docs/rag-evaluation.md</x:v>
+        <x:v>docs/ia.md / docs/찾아봇_IA_갱신본.xlsx</x:v>
       </x:c>
       <x:c r="C9" s="14" t="str">
-        <x:v>교수 피드백 반영 평가 설계</x:v>
+        <x:v>구현 기준 IA 정리</x:v>
       </x:c>
       <x:c r="D9" s="14" t="str">
-        <x:v>ROUGE/METEOR/BERTScore/Faithfulness 방향을 반영한 예비 평가 화면을 구현하였다.</x:v>
+        <x:v>기획 IA를 개발 구현 기준으로 갱신하였다.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="43.5" customHeight="1">
       <x:c r="A10" s="14" t="str">
-        <x:v>음성 설계 문서</x:v>
+        <x:v>RAG 평가 문서</x:v>
       </x:c>
       <x:c r="B10" s="14" t="str">
-        <x:v>docs/voice-architecture.md</x:v>
+        <x:v>docs/rag-evaluation.md</x:v>
       </x:c>
       <x:c r="C10" s="14" t="str">
-        <x:v>STT/TTS 및 네이버 연동 구조</x:v>
+        <x:v>교수 피드백 반영 평가 설계</x:v>
       </x:c>
       <x:c r="D10" s="14" t="str">
-        <x:v>국내 결제가 가능한 NAVER Cloud 기반 운영 버전 확장안을 설계하였다.</x:v>
+        <x:v>ROUGE/METEOR/BERTScore/Faithfulness 방향을 반영하되 사용자 화면과 분리한 내부 평가 구조를 구현하였다.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="43.5" customHeight="1">
       <x:c r="A11" s="14" t="str">
-        <x:v>선제 안부 설계</x:v>
+        <x:v>내부 평가 화면</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
-        <x:v>docs/proactive-care-plan.md</x:v>
+        <x:v>admin.html / admin.js</x:v>
       </x:c>
       <x:c r="C11" s="14" t="str">
-        <x:v>찾아봇이 먼저 말 거는 기능 기획</x:v>
+        <x:v>RAG·검색 평가 실행 및 JSON 다운로드</x:v>
       </x:c>
       <x:c r="D11" s="14" t="str">
-        <x:v>어르신에게 먼저 안부를 묻는 선제형 대화 구조를 설계하였다.</x:v>
+        <x:v>AI/알고리즘 평가는 사용자 프로토타입이 아닌 관리자 화면에서 수행하도록 분리하였다.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="43.5" customHeight="1">
       <x:c r="A12" s="14" t="str">
-        <x:v>Vercel 설정</x:v>
+        <x:v>음성 설계 문서</x:v>
       </x:c>
       <x:c r="B12" s="14" t="str">
-        <x:v>vercel.json</x:v>
+        <x:v>docs/voice-architecture.md</x:v>
       </x:c>
       <x:c r="C12" s="14" t="str">
-        <x:v>정적 배포 준비</x:v>
+        <x:v>STT/TTS 및 네이버 연동 구조</x:v>
       </x:c>
       <x:c r="D12" s="14" t="str">
-        <x:v>GitHub 연동 후 Vercel에서 즉시 배포 가능한 구조로 정리하였다.</x:v>
+        <x:v>국내 결제가 가능한 NAVER Cloud 기반 운영 버전 확장안을 설계하였다.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="43.5" customHeight="1">
       <x:c r="A13" s="14" t="str">
+        <x:v>선제 안부 설계</x:v>
+      </x:c>
+      <x:c r="B13" s="14" t="str">
+        <x:v>docs/proactive-care-plan.md</x:v>
+      </x:c>
+      <x:c r="C13" s="14" t="str">
+        <x:v>찾아봇이 먼저 말 거는 기능 기획</x:v>
+      </x:c>
+      <x:c r="D13" s="14" t="str">
+        <x:v>어르신에게 먼저 안부를 묻는 선제형 대화 구조를 설계하였다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="43.5" customHeight="1">
+      <x:c r="A14" s="14" t="str">
+        <x:v>Vercel 설정</x:v>
+      </x:c>
+      <x:c r="B14" s="14" t="str">
+        <x:v>vercel.json</x:v>
+      </x:c>
+      <x:c r="C14" s="14" t="str">
+        <x:v>정적 배포 준비</x:v>
+      </x:c>
+      <x:c r="D14" s="14" t="str">
+        <x:v>GitHub 연동 후 Vercel에서 즉시 배포 가능한 구조로 정리하였다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="43.5" customHeight="1">
+      <x:c r="A15" s="14" t="str">
         <x:v>Git 커밋</x:v>
       </x:c>
-      <x:c r="B13" s="14" t="str">
+      <x:c r="B15" s="14" t="str">
         <x:v>96e7dc4 Add Chajabot voice-enabled MVP</x:v>
       </x:c>
-      <x:c r="C13" s="14" t="str">
+      <x:c r="C15" s="14" t="str">
         <x:v>개발 이력 증빙</x:v>
       </x:c>
-      <x:c r="D13" s="14" t="str">
+      <x:c r="D15" s="14" t="str">
         <x:v>개발 산출물을 Git 커밋으로 관리하였다.</x:v>
       </x:c>
     </x:row>

</xml_diff>